<commit_message>
Move second count of pharmacy 16 to Sep 14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/مستحقات جرد الصيدليات 2026.xlsx
+++ b/inventory/مستحقات جرد الصيدليات 2026.xlsx
@@ -731,12 +731,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>الأحد</t>
+          <t>الاثنين</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -774,12 +774,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>الأحد</t>
+          <t>الاثنين</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -813,12 +813,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>الأحد</t>
+          <t>الاثنين</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -852,12 +852,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>الأحد</t>
+          <t>الاثنين</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">

</xml_diff>